<commit_message>
governance: lock approved multi-surface execution authority
</commit_message>
<xml_diff>
--- a/output/final-audit-2026-09-21/LUMENIS_MISSING_CAPABILITY_REGISTER_2026-09-21.xlsx
+++ b/output/final-audit-2026-09-21/LUMENIS_MISSING_CAPABILITY_REGISTER_2026-09-21.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="缺失总表" sheetId="1" r:id="R1e1627b852ab4c2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="44屏覆盖" sheetId="2" r:id="R9ff18bd914c44186"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="能力源码矩阵" sheetId="3" r:id="Racd9c7a78dfb460c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15轮" sheetId="4" r:id="R181d3698515c47d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PDF全覆盖" sheetId="5" r:id="R43e904e4513d435d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="6" r:id="Raba121a1cbf144d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="状态定义" sheetId="7" r:id="R8ed338b947e74ac9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="缺失总表" sheetId="1" r:id="R73b221d33c144c9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="44屏覆盖" sheetId="2" r:id="Rcf3fa903b9cf48cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="能力源码矩阵" sheetId="3" r:id="R47b49e826c894434"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15轮" sheetId="4" r:id="R07031c76b99246c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PDF全覆盖" sheetId="5" r:id="Rd1faef4665794107"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="6" r:id="R76ac8686102d470e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="状态定义" sheetId="7" r:id="R4b76b4be7c4e4f4d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -738,7 +738,7 @@
       </x:c>
       <x:c r="E5" s="11" t="n">
         <x:f>COUNTIF(E8:E47,"PARTIAL")</x:f>
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F5" s="11" t="n">
         <x:f>COUNTIF(E8:E47,"BLOCKED")</x:f>
@@ -1637,16 +1637,16 @@
         <x:v>Governance drift</x:v>
       </x:c>
       <x:c r="D30" s="26" t="str">
-        <x:v>Product positioning still describes app-only endpoints</x:v>
+        <x:v>Product positioning previously described app-only endpoints</x:v>
       </x:c>
       <x:c r="E30" s="26" t="str">
-        <x:v>PARTIAL</x:v>
+        <x:v>TESTED</x:v>
       </x:c>
       <x:c r="F30" s="26" t="str">
-        <x:v>PRODUCT-POSITIONING-CURRENT.md omits Public Website/Web Workspace</x:v>
+        <x:v>PRODUCT-POSITIONING-CURRENT.md now records Public Website/Web Workspace/Desktop/Mobile and the blocking Only-One validator requires them</x:v>
       </x:c>
       <x:c r="G30" s="26" t="str">
-        <x:v>Reconcile in Round 02 without creating second authority</x:v>
+        <x:v>Preserve the approved four-surface wording; implementation remains assigned to its scheduled rounds</x:v>
       </x:c>
       <x:c r="H30" s="26" t="str">
         <x:v>Sol / Product Architecture</x:v>
@@ -1658,10 +1658,10 @@
         <x:v>000–005, 019</x:v>
       </x:c>
       <x:c r="K30" s="26" t="str">
-        <x:v>All current authorities and validators state four surfaces consistently</x:v>
+        <x:v>Current authorities and validators state four surfaces consistently; absent runtime surfaces are not reported as implemented</x:v>
       </x:c>
       <x:c r="L30" s="26" t="str">
-        <x:v>PO reviews this audit</x:v>
+        <x:v>Architecture approved; no implementation claim</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">
@@ -1675,16 +1675,16 @@
         <x:v>Launch path drift</x:v>
       </x:c>
       <x:c r="D31" s="26" t="str">
-        <x:v>Launch plan references broader D:\LUMENIS_REBUILD path</x:v>
+        <x:v>Launch plan previously referenced the broader D:\LUMENIS_REBUILD path</x:v>
       </x:c>
       <x:c r="E31" s="26" t="str">
-        <x:v>PARTIAL</x:v>
+        <x:v>TESTED</x:v>
       </x:c>
       <x:c r="F31" s="26" t="str">
-        <x:v>LAUNCH-CONVERGENCE-MASTER-PLAN-V1.md vs canonical repo path</x:v>
+        <x:v>LAUNCH-CONVERGENCE-MASTER-PLAN-V1.md is now a subordinate Round 15 gate and resolves D:\LUMENIS_REBUILD\序\序境</x:v>
       </x:c>
       <x:c r="G31" s="26" t="str">
-        <x:v>Correct authority pointers after approval</x:v>
+        <x:v>Preserve the canonical path and subordinate launch-gate role</x:v>
       </x:c>
       <x:c r="H31" s="26" t="str">
         <x:v>Sol / Runtime</x:v>
@@ -1696,7 +1696,7 @@
         <x:v>017, 019</x:v>
       </x:c>
       <x:c r="K31" s="26" t="str">
-        <x:v>All launch/runbooks resolve canonical repo and actual entrypoint</x:v>
+        <x:v>All launch/runbooks resolve the canonical repository and actual entrypoint</x:v>
       </x:c>
       <x:c r="L31" s="26" t="str">
         <x:v>No relocation</x:v>
@@ -2326,7 +2326,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9d95b069ae243e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68dd562c136d4934"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4935,7 +4935,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra67d5cafac414d34"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf514ca494bc34426"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7881,7 +7881,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R048a2e6157da4436"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b416f1312cb414a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8554,7 +8554,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfacacaae001b448a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfffc109c2d4a48cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19250,7 +19250,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R630d64d2fb52481a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16f28a7bde0c4c49"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19557,7 +19557,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e6ded92fa5e40bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12fc657f1bba42ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19738,7 +19738,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71280a81ee844bdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R180857476c2142ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: refresh approved round 01 delivery evidence
</commit_message>
<xml_diff>
--- a/output/final-audit-2026-09-21/LUMENIS_MISSING_CAPABILITY_REGISTER_2026-09-21.xlsx
+++ b/output/final-audit-2026-09-21/LUMENIS_MISSING_CAPABILITY_REGISTER_2026-09-21.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="缺失总表" sheetId="1" r:id="R73b221d33c144c9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="44屏覆盖" sheetId="2" r:id="Rcf3fa903b9cf48cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="能力源码矩阵" sheetId="3" r:id="R47b49e826c894434"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15轮" sheetId="4" r:id="R07031c76b99246c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PDF全覆盖" sheetId="5" r:id="Rd1faef4665794107"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="6" r:id="R76ac8686102d470e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="状态定义" sheetId="7" r:id="R4b76b4be7c4e4f4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="缺失总表" sheetId="1" r:id="R31c1567afa234a2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="44屏覆盖" sheetId="2" r:id="R0f8c26cbaa7c47dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="能力源码矩阵" sheetId="3" r:id="Reb6ac61045874078"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15轮" sheetId="4" r:id="R1b7f810a45bd442d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PDF全覆盖" sheetId="5" r:id="R19fca5de01394a5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="6" r:id="R2d9a5f10e14945e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="状态定义" sheetId="7" r:id="Rb33447265b7b4f32"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1111,10 +1111,10 @@
         <x:v>BLOCKED</x:v>
       </x:c>
       <x:c r="F16" s="26" t="str">
-        <x:v>Latest runs at 3f93c128 failed before any steps; current df15a99d has no run</x:v>
+        <x:v>Current-head Product/App jobs were created but GitHub did not start any steps: recent account payments failed or the spending limit must be increased</x:v>
       </x:c>
       <x:c r="G16" s="26" t="str">
-        <x:v>Repair runner/account/infrastructure and execute current-head blocking gates</x:v>
+        <x:v>Repair GitHub billing/spending-limit availability, then rerun both current-head blocking gates</x:v>
       </x:c>
       <x:c r="H16" s="26" t="str">
         <x:v>SYSTEM Release</x:v>
@@ -1129,7 +1129,7 @@
         <x:v>Current SHA has complete logs and green required jobs; Tier C remains separate</x:v>
       </x:c>
       <x:c r="L16" s="26" t="str">
-        <x:v>May require GitHub billing/runner action</x:v>
+        <x:v>Requires GitHub billing/spending-limit action</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
@@ -2326,7 +2326,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68dd562c136d4934"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf04aa7d8b87c474b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4935,7 +4935,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf514ca494bc34426"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80d04f49c4124a4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7881,7 +7881,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b416f1312cb414a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4525292297734c13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8554,7 +8554,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfffc109c2d4a48cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R066d24e0a584463a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19250,7 +19250,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16f28a7bde0c4c49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0487d61beeb54f9e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19538,7 +19538,7 @@
         <x:v>GitHub gates</x:v>
       </x:c>
       <x:c r="C16" s="26" t="str">
-        <x:v>NOT RUN / latest attempted jobs failed before steps</x:v>
+        <x:v>BLOCKED / GitHub billing or spending limit prevented all job steps</x:v>
       </x:c>
       <x:c r="D16" s="26" t="str">
         <x:v>workflow/run inspection</x:v>
@@ -19557,7 +19557,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12fc657f1bba42ed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3febbe48beee4b94"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19738,7 +19738,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R180857476c2142ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5bd7af2d1de4395"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>